<commit_message>
Update demo downsampling to high-genotype (read_count>100) reads
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/rep1_startWT_E_demo/output/sample_results.xlsx
+++ b/demo/rep1_startWT_E_demo/output/sample_results.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H2" t="n">
         <v>-0</v>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -586,7 +586,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Demo: retain all reads for high-abundance plotted genotypes
Replace md5 1/10 subsampling with reads that map to up to the ten
highest-read-count genotypes on plotted_mutation_sets with read_count
>100 (full 1-48_C4_n27 analysis); rep1 WT/E has only five such rows, so
all five are included with every mapped read.

New demo input: input_demo_plotted_genotypes_all_reads.fa plus
demo_selected_genotypes.txt. Rerun analysis and refresh expected hashes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/rep1_startWT_E_demo/output/sample_results.xlsx
+++ b/demo/rep1_startWT_E_demo/output/sample_results.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,16 +492,48 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>135</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0.08726567550096961</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
+        <v>1547</v>
       </c>
       <c r="H2" t="n">
-        <v>-0</v>
+        <v>1.993560802313463</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sp24</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>WT-specific</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1412</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9127343244990304</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1547</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.993560802313463</v>
       </c>
     </row>
   </sheetData>
@@ -515,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,11 +574,71 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>135</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>starting_sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>K225I</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>603</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WT-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>K225L</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>529</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>WT-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>G220V; K225I</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>141</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>WT-specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>K225T</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>139</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>WT-specific</t>
         </is>
       </c>
     </row>
@@ -561,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,10 +678,32 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>135</v>
       </c>
       <c r="C2" t="n">
+        <v>0.08726567550096961</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>742</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.4796380090497738</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>670</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.4330963154492566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>